<commit_message>
Presentación oficial entrega 26 mayo 2026 - Instelec
- Actualizar presentación_entrega.html con 9 slides ejecutivas
- Incluye: resumen, 10 módulos, 6 indicadores, stack tecnológico, logros, roadmap
- Actualizar documentación de Excel e indicadores para delivery
- Listo para entrega oficial

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentacion/INDICADORES CONSTRUCCION.xlsx
+++ b/Documentacion/INDICADORES CONSTRUCCION.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Catherine Parra\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anaso\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4032961B-6CBD-4C3C-A12C-FC49DFBD8494}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FDA9434-36E2-4D0A-9DE5-4578AF386DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="870" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="870" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="8" r:id="rId1"/>
@@ -21,6 +21,19 @@
     <externalReference r:id="rId4"/>
   </externalReferences>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -114,21 +127,12 @@
   <commentList>
     <comment ref="F10" authorId="0" shapeId="0" xr:uid="{3FB8D28C-33B4-477E-B02B-BA5C886B270C}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">[Comentario encadenado]
-Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
+        <t xml:space="preserve">[Comentario encadenado]
+Tu versión de Excel te permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
 Comentario:
     $ 139.962.400
 PRESTAMO JUANCHOANITA
 </t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -1089,7 +1093,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -2109,7 +2113,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -3545,7 +3549,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="es-ES"/>
+  <c:lang val="es-MX"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -6009,7 +6013,7 @@
               <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="'[1]973'!$F$494:$G$496" spid="_x0000_s1249"/>
+                  <a14:cameraTool cellRange="'[1]973'!$F$494:$G$496" spid="_x0000_s1250"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -6802,25 +6806,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96817F0B-C9C3-4D89-817B-DA33BF968DE9}">
   <dimension ref="A16:P147"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="28.109375" customWidth="1"/>
-    <col min="12" max="13" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.88671875" customWidth="1"/>
-    <col min="15" max="15" width="16.88671875" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28.140625" customWidth="1"/>
+    <col min="12" max="13" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.85546875" customWidth="1"/>
+    <col min="15" max="15" width="16.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="16" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:8" x14ac:dyDescent="0.25">
       <c r="C16" s="4" t="s">
         <v>24</v>
       </c>
@@ -6837,7 +6841,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="3:15" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
         <v>2</v>
       </c>
@@ -6852,7 +6856,7 @@
         <v>6343795930</v>
       </c>
     </row>
-    <row r="18" spans="3:15" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
         <v>3</v>
       </c>
@@ -6862,7 +6866,7 @@
       <c r="F18" s="8"/>
       <c r="G18" s="8"/>
     </row>
-    <row r="19" spans="3:15" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
         <v>7</v>
       </c>
@@ -6872,7 +6876,7 @@
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
     </row>
-    <row r="20" spans="3:15" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
         <v>8</v>
       </c>
@@ -6882,7 +6886,7 @@
       <c r="F20" s="8"/>
       <c r="G20" s="8"/>
     </row>
-    <row r="21" spans="3:15" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C21" s="4" t="s">
         <v>9</v>
       </c>
@@ -6899,7 +6903,7 @@
       </c>
       <c r="O21" s="5"/>
     </row>
-    <row r="22" spans="3:15" s="7" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:15" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="C22" s="7" t="s">
         <v>10</v>
       </c>
@@ -6917,7 +6921,7 @@
       </c>
       <c r="O22" s="6"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C38" s="95" t="s">
         <v>24</v>
       </c>
@@ -6932,7 +6936,7 @@
       <c r="J38" s="94"/>
       <c r="K38" s="94"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2024</v>
       </c>
@@ -6963,7 +6967,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="8">
         <v>2423118863</v>
       </c>
@@ -7005,7 +7009,7 @@
         <v>0.73197645349999996</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>12</v>
       </c>
@@ -7033,7 +7037,7 @@
       </c>
       <c r="L41" s="3"/>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>13</v>
       </c>
@@ -7061,7 +7065,7 @@
       </c>
       <c r="L42" s="3"/>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
         <v>14</v>
       </c>
@@ -7094,7 +7098,7 @@
         <v>0.1152063664</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>17</v>
       </c>
@@ -7121,7 +7125,7 @@
         <v>0.12693147483333334</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>18</v>
       </c>
@@ -7160,7 +7164,7 @@
         <v>2.5885705266666666E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B46" s="4" t="s">
         <v>4</v>
       </c>
@@ -7200,7 +7204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G47" s="20"/>
       <c r="H47" s="21"/>
       <c r="I47" s="21"/>
@@ -7209,7 +7213,7 @@
         <v>30000000000</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B48" s="4" t="s">
         <v>15</v>
       </c>
@@ -7246,7 +7250,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="49" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B49" t="s">
         <v>11</v>
       </c>
@@ -7281,7 +7285,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="50" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B50" t="s">
         <v>14</v>
       </c>
@@ -7293,7 +7297,7 @@
         <v>3456190.9920000001</v>
       </c>
     </row>
-    <row r="51" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B51" t="s">
         <v>17</v>
       </c>
@@ -7303,7 +7307,7 @@
         <v>3807944.2450000001</v>
       </c>
     </row>
-    <row r="52" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B52" t="s">
         <v>19</v>
       </c>
@@ -7313,7 +7317,7 @@
         <v>776571.15799999889</v>
       </c>
     </row>
-    <row r="53" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B53" s="4" t="s">
         <v>4</v>
       </c>
@@ -7325,12 +7329,12 @@
         <v>30000000</v>
       </c>
     </row>
-    <row r="54" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:15" x14ac:dyDescent="0.25">
       <c r="D54" s="15">
         <v>30000000</v>
       </c>
     </row>
-    <row r="58" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:15" x14ac:dyDescent="0.25">
       <c r="L58" s="2"/>
       <c r="N58" s="8">
         <v>335737310</v>
@@ -7339,7 +7343,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:15" x14ac:dyDescent="0.25">
       <c r="L59" s="2"/>
       <c r="N59" s="8">
         <v>498947535</v>
@@ -7348,7 +7352,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="60" spans="2:15" x14ac:dyDescent="0.25">
       <c r="L60" s="2"/>
       <c r="N60" s="8">
         <v>344584158</v>
@@ -7357,7 +7361,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:15" x14ac:dyDescent="0.25">
       <c r="L61" s="2"/>
       <c r="N61" s="8">
         <v>288975890</v>
@@ -7366,7 +7370,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="62" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:15" x14ac:dyDescent="0.25">
       <c r="L62" s="2"/>
       <c r="N62" s="8">
         <v>507923325</v>
@@ -7375,7 +7379,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="63" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:15" x14ac:dyDescent="0.25">
       <c r="L63" s="2"/>
       <c r="N63" s="8">
         <v>406480130</v>
@@ -7384,7 +7388,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="64" spans="2:15" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:15" x14ac:dyDescent="0.25">
       <c r="L64" s="2"/>
       <c r="N64" s="8">
         <v>1171614120</v>
@@ -7393,7 +7397,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="11:15" x14ac:dyDescent="0.3">
+    <row r="65" spans="11:15" x14ac:dyDescent="0.25">
       <c r="L65" s="2"/>
       <c r="N65" s="8">
         <v>253681777</v>
@@ -7402,7 +7406,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="66" spans="11:15" x14ac:dyDescent="0.3">
+    <row r="66" spans="11:15" x14ac:dyDescent="0.25">
       <c r="L66" s="5" t="s">
         <v>16</v>
       </c>
@@ -7412,7 +7416,7 @@
       </c>
       <c r="O66"/>
     </row>
-    <row r="75" spans="11:15" x14ac:dyDescent="0.3">
+    <row r="75" spans="11:15" x14ac:dyDescent="0.25">
       <c r="K75" s="4" t="s">
         <v>25</v>
       </c>
@@ -7423,7 +7427,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="76" spans="11:15" x14ac:dyDescent="0.3">
+    <row r="76" spans="11:15" x14ac:dyDescent="0.25">
       <c r="K76" s="8">
         <v>-11046360810.92</v>
       </c>
@@ -7435,7 +7439,7 @@
         <v>-6039486169.8199997</v>
       </c>
     </row>
-    <row r="77" spans="11:15" x14ac:dyDescent="0.3">
+    <row r="77" spans="11:15" x14ac:dyDescent="0.25">
       <c r="K77" s="8">
         <v>3835241765.0999999</v>
       </c>
@@ -7447,7 +7451,7 @@
         <v>1320606819.54</v>
       </c>
     </row>
-    <row r="78" spans="11:15" x14ac:dyDescent="0.3">
+    <row r="78" spans="11:15" x14ac:dyDescent="0.25">
       <c r="K78" s="8">
         <v>787323995.42999995</v>
       </c>
@@ -7459,7 +7463,7 @@
         <v>636145394.20999992</v>
       </c>
     </row>
-    <row r="79" spans="11:15" x14ac:dyDescent="0.3">
+    <row r="79" spans="11:15" x14ac:dyDescent="0.25">
       <c r="K79" s="8">
         <v>9532785831.2199993</v>
       </c>
@@ -7471,7 +7475,7 @@
         <v>6393257465.6799994</v>
       </c>
     </row>
-    <row r="80" spans="11:15" x14ac:dyDescent="0.3">
+    <row r="80" spans="11:15" x14ac:dyDescent="0.25">
       <c r="K80" s="9">
         <f>+SUM(K76:K79)</f>
         <v>3108990780.8299999</v>
@@ -7485,7 +7489,7 @@
         <v>2310523509.6099997</v>
       </c>
     </row>
-    <row r="81" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="81" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K81" s="10">
         <f>+K80/K76</f>
         <v>-0.28144932381319404</v>
@@ -7499,12 +7503,12 @@
         <v>-0.38256955056142833</v>
       </c>
     </row>
-    <row r="82" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="82" spans="11:14" x14ac:dyDescent="0.25">
       <c r="N82" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="83" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="83" spans="11:14" x14ac:dyDescent="0.25">
       <c r="M83" s="8">
         <f>(327073712+641955838+850560874)-(327073712+641955838)</f>
         <v>850560874</v>
@@ -7513,7 +7517,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="119" spans="11:16" x14ac:dyDescent="0.3">
+    <row r="119" spans="11:16" x14ac:dyDescent="0.25">
       <c r="L119" s="12" t="s">
         <v>5</v>
       </c>
@@ -7530,7 +7534,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="120" spans="11:16" x14ac:dyDescent="0.3">
+    <row r="120" spans="11:16" x14ac:dyDescent="0.25">
       <c r="K120" t="s">
         <v>2</v>
       </c>
@@ -7549,7 +7553,7 @@
         <v>-11061884416.16</v>
       </c>
     </row>
-    <row r="121" spans="11:16" x14ac:dyDescent="0.3">
+    <row r="121" spans="11:16" x14ac:dyDescent="0.25">
       <c r="K121" t="s">
         <v>26</v>
       </c>
@@ -7570,7 +7574,7 @@
         <v>2702575271.96</v>
       </c>
     </row>
-    <row r="122" spans="11:16" x14ac:dyDescent="0.3">
+    <row r="122" spans="11:16" x14ac:dyDescent="0.25">
       <c r="K122" t="s">
         <v>27</v>
       </c>
@@ -7589,7 +7593,7 @@
         <v>787323995.42999995</v>
       </c>
     </row>
-    <row r="123" spans="11:16" x14ac:dyDescent="0.3">
+    <row r="123" spans="11:16" x14ac:dyDescent="0.25">
       <c r="K123" t="s">
         <v>8</v>
       </c>
@@ -7610,7 +7614,7 @@
         <v>7065102796.9700012</v>
       </c>
     </row>
-    <row r="124" spans="11:16" x14ac:dyDescent="0.3">
+    <row r="124" spans="11:16" x14ac:dyDescent="0.25">
       <c r="K124" s="4" t="s">
         <v>9</v>
       </c>
@@ -7635,7 +7639,7 @@
         <v>-506882351.79999828</v>
       </c>
     </row>
-    <row r="125" spans="11:16" x14ac:dyDescent="0.3">
+    <row r="125" spans="11:16" x14ac:dyDescent="0.25">
       <c r="L125" s="10">
         <f>+L124/L120</f>
         <v>-0.21259866733674421</v>
@@ -7652,7 +7656,7 @@
         <v>498978093.99999964</v>
       </c>
     </row>
-    <row r="126" spans="11:16" x14ac:dyDescent="0.3">
+    <row r="126" spans="11:16" x14ac:dyDescent="0.25">
       <c r="K126" t="s">
         <v>31</v>
       </c>
@@ -7675,7 +7679,7 @@
         <v>-7904257.799998641</v>
       </c>
     </row>
-    <row r="127" spans="11:16" x14ac:dyDescent="0.3">
+    <row r="127" spans="11:16" x14ac:dyDescent="0.25">
       <c r="K127" s="4" t="s">
         <v>32</v>
       </c>
@@ -7696,7 +7700,7 @@
         <v>-0.49903039436720298</v>
       </c>
     </row>
-    <row r="128" spans="11:16" x14ac:dyDescent="0.3">
+    <row r="128" spans="11:16" x14ac:dyDescent="0.25">
       <c r="L128" s="10">
         <f>+L127/L120</f>
         <v>0.18083677618121469</v>
@@ -7710,7 +7714,7 @@
         <v>-0.10166558401361392</v>
       </c>
     </row>
-    <row r="129" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="129" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K129" t="s">
         <v>95</v>
       </c>
@@ -7727,7 +7731,7 @@
         <v>-4514940681</v>
       </c>
     </row>
-    <row r="130" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="130" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K130" s="4" t="s">
         <v>107</v>
       </c>
@@ -7744,7 +7748,7 @@
         <v>-3390327741.539999</v>
       </c>
     </row>
-    <row r="131" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="131" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K131" s="86" t="s">
         <v>108</v>
       </c>
@@ -7761,7 +7765,7 @@
         <v>0.21765203887139561</v>
       </c>
     </row>
-    <row r="133" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="133" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K133" s="4" t="s">
         <v>106</v>
       </c>
@@ -7772,7 +7776,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="134" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="134" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K134" t="s">
         <v>97</v>
       </c>
@@ -7780,7 +7784,7 @@
         <v>73338.929999999993</v>
       </c>
     </row>
-    <row r="135" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="135" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K135" s="79" t="s">
         <v>99</v>
       </c>
@@ -7788,7 +7792,7 @@
         <v>1137010315.4400001</v>
       </c>
     </row>
-    <row r="136" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="136" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K136" t="s">
         <v>98</v>
       </c>
@@ -7796,7 +7800,7 @@
         <v>803084066.95000005</v>
       </c>
     </row>
-    <row r="137" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="137" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K137" s="82" t="s">
         <v>104</v>
       </c>
@@ -7806,7 +7810,7 @@
         <v>1940167721.3200002</v>
       </c>
     </row>
-    <row r="138" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="138" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K138" t="s">
         <v>100</v>
       </c>
@@ -7814,7 +7818,7 @@
         <v>1260023331.4300001</v>
       </c>
     </row>
-    <row r="139" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="139" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K139" s="82" t="s">
         <v>101</v>
       </c>
@@ -7824,7 +7828,7 @@
         <v>3200191052.75</v>
       </c>
     </row>
-    <row r="140" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="140" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K140" s="80" t="s">
         <v>102</v>
       </c>
@@ -7834,7 +7838,7 @@
         <v>1260023331.4299998</v>
       </c>
     </row>
-    <row r="141" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="141" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K141" t="s">
         <v>91</v>
       </c>
@@ -7846,7 +7850,7 @@
         <v>1372455859.75</v>
       </c>
     </row>
-    <row r="142" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="142" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K142" t="s">
         <v>92</v>
       </c>
@@ -7857,7 +7861,7 @@
         <v>1921965210</v>
       </c>
     </row>
-    <row r="143" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="143" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K143" s="82" t="s">
         <v>105</v>
       </c>
@@ -7870,7 +7874,7 @@
         <v>4554444401.1800003</v>
       </c>
     </row>
-    <row r="144" spans="11:14" x14ac:dyDescent="0.3">
+    <row r="144" spans="11:14" x14ac:dyDescent="0.25">
       <c r="K144" t="s">
         <v>93</v>
       </c>
@@ -7881,7 +7885,7 @@
         <v>3775322530</v>
       </c>
     </row>
-    <row r="145" spans="11:13" x14ac:dyDescent="0.3">
+    <row r="145" spans="11:13" x14ac:dyDescent="0.25">
       <c r="K145" s="82" t="s">
         <v>94</v>
       </c>
@@ -7894,7 +7898,7 @@
         <v>7069743599.75</v>
       </c>
     </row>
-    <row r="146" spans="11:13" x14ac:dyDescent="0.3">
+    <row r="146" spans="11:13" x14ac:dyDescent="0.25">
       <c r="K146" s="80" t="s">
         <v>103</v>
       </c>
@@ -7907,7 +7911,7 @@
         <v>2515299198.5699997</v>
       </c>
     </row>
-    <row r="147" spans="11:13" x14ac:dyDescent="0.3">
+    <row r="147" spans="11:13" x14ac:dyDescent="0.25">
       <c r="M147" s="31"/>
     </row>
   </sheetData>
@@ -7924,26 +7928,26 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B8D58E6-15CC-4296-9B80-6262277DC854}">
   <dimension ref="A1:XFA50"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="12" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.33203125" style="39" customWidth="1"/>
+    <col min="1" max="1" width="32.28515625" style="39" customWidth="1"/>
     <col min="2" max="2" width="8" style="74" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.33203125" style="75" customWidth="1"/>
-    <col min="4" max="5" width="8.88671875" style="75" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.44140625" style="54" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6.109375" style="75" customWidth="1"/>
-    <col min="8" max="8" width="5.6640625" style="75" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="9" max="9" width="7.88671875" style="75" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="3" max="3" width="8.28515625" style="75" customWidth="1"/>
+    <col min="4" max="5" width="8.85546875" style="75" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.42578125" style="54" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.140625" style="75" customWidth="1"/>
+    <col min="8" max="8" width="5.7109375" style="75" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="9" max="9" width="7.85546875" style="75" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="10" max="10" width="11" style="75" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="11" max="13" width="10.6640625" style="75" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="14" max="14" width="11.6640625" style="75" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="15" max="15" width="6.33203125" style="43" hidden="1" customWidth="1"/>
+    <col min="11" max="13" width="10.7109375" style="75" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="14" max="14" width="11.7109375" style="75" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="15" max="15" width="6.28515625" style="43" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="7" style="43" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="14.109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="11.44140625" style="39"/>
+    <col min="17" max="17" width="14.140625" style="39" bestFit="1" customWidth="1"/>
+    <col min="18" max="16384" width="11.42578125" style="39"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="34" t="s">
         <v>33</v>
       </c>
@@ -7993,7 +7997,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="40" t="s">
         <v>49</v>
       </c>
@@ -8035,7 +8039,7 @@
       </c>
       <c r="Q2" s="44"/>
     </row>
-    <row r="3" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="45" t="s">
         <v>50</v>
       </c>
@@ -8073,7 +8077,7 @@
       </c>
       <c r="P3" s="46"/>
     </row>
-    <row r="4" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="40" t="s">
         <v>51</v>
       </c>
@@ -8115,7 +8119,7 @@
       </c>
       <c r="Q4" s="44"/>
     </row>
-    <row r="5" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" s="50" customFormat="1" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" s="50" customFormat="1" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="47" t="s">
         <v>52</v>
       </c>
@@ -9361,7 +9365,7 @@
       <c r="XEM5" s="51"/>
       <c r="XFA5" s="51"/>
     </row>
-    <row r="6" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="52"/>
       <c r="C6" s="53"/>
       <c r="D6" s="53"/>
@@ -9375,7 +9379,7 @@
       <c r="M6" s="53"/>
       <c r="N6" s="53"/>
     </row>
-    <row r="7" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="34" t="s">
         <v>53</v>
       </c>
@@ -9392,7 +9396,7 @@
       <c r="M7" s="53"/>
       <c r="N7" s="53"/>
     </row>
-    <row r="8" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="55" t="s">
         <v>54</v>
       </c>
@@ -9441,7 +9445,7 @@
         <v>0.27009061926642808</v>
       </c>
     </row>
-    <row r="9" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="55" t="s">
         <v>55</v>
       </c>
@@ -9475,7 +9479,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="55" t="s">
         <v>56</v>
       </c>
@@ -9524,7 +9528,7 @@
         <v>5.8212420074271888E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="55" t="s">
         <v>57</v>
       </c>
@@ -9573,7 +9577,7 @@
         <v>7.3873927456181876E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="55" t="s">
         <v>58</v>
       </c>
@@ -9622,7 +9626,7 @@
         <v>2.3845653695203552E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="55" t="s">
         <v>59</v>
       </c>
@@ -9671,7 +9675,7 @@
         <v>6.4229395882116944E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="55" t="s">
         <v>60</v>
       </c>
@@ -9720,7 +9724,7 @@
         <v>3.868137526657095E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="55" t="s">
         <v>61</v>
       </c>
@@ -9769,7 +9773,7 @@
         <v>4.7958714711975074E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1023 1037:2045 2059:3067 3081:4089 4103:5111 5125:6133 6147:7155 7169:8191 8205:9213 9227:10235 10249:11257 11271:12279 12293:13301 13315:14323 14337:15359 15373:16381" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="55" t="s">
         <v>62</v>
       </c>
@@ -9818,7 +9822,7 @@
         <v>5.7037696828748296E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="55" t="s">
         <v>63</v>
       </c>
@@ -9867,7 +9871,7 @@
         <v>3.0477151574969139E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="55" t="s">
         <v>64</v>
       </c>
@@ -9916,7 +9920,7 @@
         <v>1.0539881828482776E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="55" t="s">
         <v>65</v>
       </c>
@@ -9965,7 +9969,7 @@
         <v>6.2293700055514973E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="55" t="s">
         <v>66</v>
       </c>
@@ -10014,7 +10018,7 @@
         <v>7.1145331283594066E-4</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="55" t="s">
         <v>67</v>
       </c>
@@ -10063,7 +10067,7 @@
         <v>0.14546289929408085</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="55" t="s">
         <v>68</v>
       </c>
@@ -10104,7 +10108,7 @@
         <v>0.12797237642252116</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="55" t="s">
         <v>69</v>
       </c>
@@ -10149,7 +10153,7 @@
         <v>0.13905263471852067</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="58" t="s">
         <v>70</v>
       </c>
@@ -10222,7 +10226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="52"/>
       <c r="C25" s="53"/>
       <c r="D25" s="53"/>
@@ -10236,7 +10240,7 @@
       <c r="M25" s="53"/>
       <c r="N25" s="53"/>
     </row>
-    <row r="26" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="61" t="s">
         <v>71</v>
       </c>
@@ -10301,7 +10305,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="52"/>
       <c r="C27" s="53"/>
       <c r="D27" s="53"/>
@@ -10315,7 +10319,7 @@
       <c r="M27" s="53"/>
       <c r="N27" s="53"/>
     </row>
-    <row r="28" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="61" t="s">
         <v>72</v>
       </c>
@@ -10332,7 +10336,7 @@
       <c r="M28" s="53"/>
       <c r="N28" s="53"/>
     </row>
-    <row r="29" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="58" t="s">
         <v>73</v>
       </c>
@@ -10373,7 +10377,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="63"/>
       <c r="B30" s="64"/>
       <c r="C30" s="53"/>
@@ -10388,7 +10392,7 @@
       <c r="M30" s="53"/>
       <c r="N30" s="53"/>
     </row>
-    <row r="31" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="58" t="s">
         <v>74</v>
       </c>
@@ -10405,7 +10409,7 @@
       <c r="M31" s="53"/>
       <c r="N31" s="53"/>
     </row>
-    <row r="32" spans="1:18" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:18" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="66" t="s">
         <v>75</v>
       </c>
@@ -10446,7 +10450,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="33" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="66" t="s">
         <v>76</v>
       </c>
@@ -10487,7 +10491,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="66" t="s">
         <v>77</v>
       </c>
@@ -10528,7 +10532,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="67" t="s">
         <v>78</v>
       </c>
@@ -10593,7 +10597,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="52"/>
       <c r="C36" s="53"/>
       <c r="D36" s="53"/>
@@ -10607,7 +10611,7 @@
       <c r="M36" s="53"/>
       <c r="N36" s="53"/>
     </row>
-    <row r="37" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="61" t="s">
         <v>79</v>
       </c>
@@ -10672,7 +10676,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="38" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B38" s="52"/>
       <c r="C38" s="53"/>
       <c r="D38" s="53"/>
@@ -10686,7 +10690,7 @@
       <c r="M38" s="53"/>
       <c r="N38" s="53"/>
     </row>
-    <row r="39" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="61" t="s">
         <v>80</v>
       </c>
@@ -10704,7 +10708,7 @@
       <c r="M39" s="70"/>
       <c r="N39" s="70"/>
     </row>
-    <row r="40" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="72" t="s">
         <v>81</v>
       </c>
@@ -10745,7 +10749,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="41" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B41" s="52"/>
       <c r="C41" s="53"/>
       <c r="D41" s="53"/>
@@ -10759,7 +10763,7 @@
       <c r="M41" s="53"/>
       <c r="N41" s="53"/>
     </row>
-    <row r="42" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="34" t="s">
         <v>82</v>
       </c>
@@ -10824,7 +10828,7 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="43" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B43" s="52"/>
       <c r="C43" s="53"/>
       <c r="D43" s="53"/>
@@ -10838,7 +10842,7 @@
       <c r="M43" s="53"/>
       <c r="N43" s="53"/>
     </row>
-    <row r="44" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="34" t="s">
         <v>83</v>
       </c>
@@ -10885,7 +10889,7 @@
         <v>616350820.05999994</v>
       </c>
     </row>
-    <row r="45" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="34" t="s">
         <v>84</v>
       </c>
@@ -10933,7 +10937,7 @@
         <v>-269892178.73000038</v>
       </c>
     </row>
-    <row r="46" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="39" t="s">
         <v>85</v>
       </c>
@@ -10963,7 +10967,7 @@
       <c r="M46" s="53"/>
       <c r="N46" s="53"/>
     </row>
-    <row r="47" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="39" t="s">
         <v>86</v>
       </c>
@@ -10993,7 +10997,7 @@
       <c r="M47" s="53"/>
       <c r="N47" s="53"/>
     </row>
-    <row r="48" spans="1:16" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:16" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="39" t="s">
         <v>87</v>
       </c>
@@ -11019,7 +11023,7 @@
       <c r="M48" s="53"/>
       <c r="N48" s="53"/>
     </row>
-    <row r="49" spans="2:14" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:14" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="52"/>
       <c r="C49" s="53"/>
       <c r="D49" s="53"/>
@@ -11033,7 +11037,7 @@
       <c r="M49" s="52"/>
       <c r="N49" s="52"/>
     </row>
-    <row r="50" spans="2:14" ht="12.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:14" ht="12.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="52"/>
       <c r="C50" s="53"/>
       <c r="D50" s="53"/>
@@ -11056,20 +11060,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1D50E84-B22E-4225-9524-7051923059EA}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.5546875" style="93"/>
-    <col min="2" max="2" width="26.77734375" style="87" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="69.77734375" customWidth="1"/>
-    <col min="4" max="4" width="13.33203125" style="91" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.5703125" style="93"/>
+    <col min="2" max="2" width="26.7109375" style="87" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="69.7109375" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" style="91" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D1" s="90" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="68.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="68.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="93" t="s">
         <v>116</v>
       </c>
@@ -11080,7 +11084,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="93" t="s">
         <v>116</v>
       </c>
@@ -11091,7 +11095,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="54" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="93" t="s">
         <v>117</v>
       </c>
@@ -11099,7 +11103,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="52.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="52.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="93" t="s">
         <v>117</v>
       </c>
@@ -11107,7 +11111,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="93" t="s">
         <v>117</v>
       </c>
@@ -11118,8 +11122,8 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="5.4" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="5.45" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="93" t="s">
         <v>117</v>
       </c>
@@ -11127,7 +11131,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="37.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="37.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="93" t="s">
         <v>117</v>
       </c>
@@ -11138,7 +11142,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="93" t="s">
         <v>117</v>
       </c>
@@ -11152,7 +11156,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="93" t="s">
         <v>117</v>
       </c>
@@ -11166,7 +11170,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="93" t="s">
         <v>117</v>
       </c>
@@ -11180,7 +11184,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="93" t="s">
         <v>117</v>
       </c>

</xml_diff>